<commit_message>
Update .gitignore to exclude temp and OS files
</commit_message>
<xml_diff>
--- a/src/resources/testData/Test_Sheet.xlsx
+++ b/src/resources/testData/Test_Sheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Selenium\facctum-test-automation-rs_initial_test_setup\src\test\resources\testData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PlayWright-main\PlayWright-main\src\resources\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{224EDE0D-ECFF-40D1-AC63-9C7D6ADE4C8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C670506-4BC6-4371-9EA7-94D7042AC9BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Audit" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1662" uniqueCount="329">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1662" uniqueCount="328">
   <si>
     <t>FileName</t>
   </si>
@@ -1019,13 +1019,10 @@
     <t>Transaction</t>
   </si>
   <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>Transaction Screening</t>
-  </si>
-  <si>
-    <t>autoRule20</t>
+    <t>1</t>
+  </si>
+  <si>
+    <t>autoRule</t>
   </si>
 </sst>
 </file>
@@ -1413,9 +1410,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1426,7 +1423,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1449,9 +1446,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:BD25"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -1621,7 +1618,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1779,7 +1776,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="3" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1931,7 +1928,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="4" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
@@ -2077,7 +2074,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="5" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
@@ -2235,7 +2232,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="6" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>5</v>
       </c>
@@ -2393,7 +2390,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="7" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>6</v>
       </c>
@@ -2548,7 +2545,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="8" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>7</v>
       </c>
@@ -2697,7 +2694,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="9" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>8</v>
       </c>
@@ -2846,7 +2843,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="10" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>9</v>
       </c>
@@ -2995,7 +2992,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="11" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>10</v>
       </c>
@@ -3141,7 +3138,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="12" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>11</v>
       </c>
@@ -3287,7 +3284,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="13" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>12</v>
       </c>
@@ -3433,7 +3430,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="14" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>13</v>
       </c>
@@ -3591,7 +3588,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="15" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>14</v>
       </c>
@@ -3743,7 +3740,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="16" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>15</v>
       </c>
@@ -3901,7 +3898,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="17" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>16</v>
       </c>
@@ -4047,7 +4044,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="18" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>17</v>
       </c>
@@ -4205,7 +4202,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="19" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>18</v>
       </c>
@@ -4360,7 +4357,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="20" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>19</v>
       </c>
@@ -4509,7 +4506,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="21" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>20</v>
       </c>
@@ -4658,7 +4655,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="22" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>21</v>
       </c>
@@ -4807,7 +4804,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="23" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>22</v>
       </c>
@@ -4959,7 +4956,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="24" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>23</v>
       </c>
@@ -5117,7 +5114,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="25" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>24</v>
       </c>
@@ -5287,13 +5284,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9990FD1D-23E8-4132-9AD5-48C8D906EBBA}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:F85"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="3" width="11.375" customWidth="1"/>
+    <col min="3" max="3" width="11.33203125" customWidth="1"/>
     <col min="4" max="4" width="47.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>229</v>
       </c>
@@ -5313,7 +5310,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>234</v>
       </c>
@@ -5333,7 +5330,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>234</v>
       </c>
@@ -5353,7 +5350,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>234</v>
       </c>
@@ -5373,7 +5370,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>234</v>
       </c>
@@ -5393,7 +5390,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>234</v>
       </c>
@@ -5413,7 +5410,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>234</v>
       </c>
@@ -5433,7 +5430,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>234</v>
       </c>
@@ -5453,7 +5450,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>234</v>
       </c>
@@ -5473,7 +5470,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>234</v>
       </c>
@@ -5493,7 +5490,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>228</v>
       </c>
@@ -5513,7 +5510,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>228</v>
       </c>
@@ -5533,7 +5530,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>228</v>
       </c>
@@ -5553,7 +5550,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>228</v>
       </c>
@@ -5573,7 +5570,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>228</v>
       </c>
@@ -5593,7 +5590,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>228</v>
       </c>
@@ -5613,7 +5610,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>228</v>
       </c>
@@ -5633,7 +5630,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>228</v>
       </c>
@@ -5653,7 +5650,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>228</v>
       </c>
@@ -5673,7 +5670,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>228</v>
       </c>
@@ -5693,7 +5690,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>228</v>
       </c>
@@ -5713,7 +5710,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>228</v>
       </c>
@@ -5733,7 +5730,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>228</v>
       </c>
@@ -5753,7 +5750,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>228</v>
       </c>
@@ -5773,7 +5770,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>228</v>
       </c>
@@ -5793,7 +5790,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>228</v>
       </c>
@@ -5813,7 +5810,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>228</v>
       </c>
@@ -5833,7 +5830,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>228</v>
       </c>
@@ -5853,7 +5850,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>228</v>
       </c>
@@ -5873,7 +5870,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>228</v>
       </c>
@@ -5893,7 +5890,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>228</v>
       </c>
@@ -5913,7 +5910,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>228</v>
       </c>
@@ -5933,7 +5930,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>228</v>
       </c>
@@ -5953,7 +5950,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>228</v>
       </c>
@@ -5973,7 +5970,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>228</v>
       </c>
@@ -5993,7 +5990,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>228</v>
       </c>
@@ -6013,7 +6010,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>228</v>
       </c>
@@ -6033,7 +6030,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>228</v>
       </c>
@@ -6053,7 +6050,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>228</v>
       </c>
@@ -6073,7 +6070,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
         <v>228</v>
       </c>
@@ -6093,7 +6090,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>228</v>
       </c>
@@ -6113,7 +6110,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
         <v>228</v>
       </c>
@@ -6133,7 +6130,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
         <v>228</v>
       </c>
@@ -6153,7 +6150,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>228</v>
       </c>
@@ -6173,7 +6170,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>228</v>
       </c>
@@ -6193,7 +6190,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
         <v>228</v>
       </c>
@@ -6213,7 +6210,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>228</v>
       </c>
@@ -6233,7 +6230,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>228</v>
       </c>
@@ -6253,7 +6250,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>228</v>
       </c>
@@ -6273,7 +6270,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
         <v>228</v>
       </c>
@@ -6293,7 +6290,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
         <v>228</v>
       </c>
@@ -6313,7 +6310,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
         <v>228</v>
       </c>
@@ -6333,7 +6330,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
         <v>228</v>
       </c>
@@ -6353,7 +6350,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
         <v>228</v>
       </c>
@@ -6373,7 +6370,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
         <v>228</v>
       </c>
@@ -6393,7 +6390,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>228</v>
       </c>
@@ -6413,7 +6410,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
         <v>228</v>
       </c>
@@ -6433,7 +6430,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
         <v>228</v>
       </c>
@@ -6453,7 +6450,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>228</v>
       </c>
@@ -6473,7 +6470,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
         <v>228</v>
       </c>
@@ -6493,7 +6490,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
         <v>228</v>
       </c>
@@ -6513,7 +6510,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
         <v>228</v>
       </c>
@@ -6533,7 +6530,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63" s="1" t="s">
         <v>228</v>
       </c>
@@ -6553,7 +6550,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64" s="1" t="s">
         <v>228</v>
       </c>
@@ -6573,7 +6570,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" s="1" t="s">
         <v>228</v>
       </c>
@@ -6593,7 +6590,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" s="1" t="s">
         <v>228</v>
       </c>
@@ -6613,7 +6610,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" s="1" t="s">
         <v>228</v>
       </c>
@@ -6633,7 +6630,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A68" s="1" t="s">
         <v>228</v>
       </c>
@@ -6653,7 +6650,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A69" s="1" t="s">
         <v>228</v>
       </c>
@@ -6673,7 +6670,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A70" s="1" t="s">
         <v>228</v>
       </c>
@@ -6693,7 +6690,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A71" s="1" t="s">
         <v>228</v>
       </c>
@@ -6713,7 +6710,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72" s="1" t="s">
         <v>228</v>
       </c>
@@ -6733,7 +6730,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A73" s="1" t="s">
         <v>228</v>
       </c>
@@ -6753,7 +6750,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74" s="1" t="s">
         <v>228</v>
       </c>
@@ -6773,7 +6770,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A75" s="1" t="s">
         <v>228</v>
       </c>
@@ -6793,7 +6790,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A76" s="1" t="s">
         <v>228</v>
       </c>
@@ -6813,7 +6810,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A77" s="1" t="s">
         <v>228</v>
       </c>
@@ -6833,7 +6830,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A78" s="1" t="s">
         <v>228</v>
       </c>
@@ -6853,7 +6850,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A79" s="1" t="s">
         <v>228</v>
       </c>
@@ -6873,7 +6870,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A80" s="1" t="s">
         <v>228</v>
       </c>
@@ -6893,7 +6890,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A81" s="1" t="s">
         <v>228</v>
       </c>
@@ -6913,7 +6910,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A82" s="1" t="s">
         <v>228</v>
       </c>
@@ -6933,7 +6930,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A83" s="1" t="s">
         <v>228</v>
       </c>
@@ -6953,7 +6950,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A84" s="1" t="s">
         <v>228</v>
       </c>
@@ -6973,7 +6970,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A85" s="1" t="s">
         <v>228</v>
       </c>
@@ -7004,9 +7001,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B7ACFE9-6D4A-4EEC-B4BF-F48097A5BD6C}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:I85"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1">
         <v>95</v>
       </c>
@@ -7028,7 +7025,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>95</v>
       </c>
@@ -7057,7 +7054,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>95</v>
       </c>
@@ -7082,7 +7079,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>95</v>
       </c>
@@ -7107,7 +7104,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>95</v>
       </c>
@@ -7132,7 +7129,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>90</v>
       </c>
@@ -7157,7 +7154,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>84</v>
       </c>
@@ -7182,7 +7179,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>84</v>
       </c>
@@ -7207,7 +7204,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>83</v>
       </c>
@@ -7232,7 +7229,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="F10" s="1">
         <v>81</v>
       </c>
@@ -7243,7 +7240,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="F11" s="1">
         <v>98</v>
       </c>
@@ -7254,7 +7251,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="F12" s="1">
         <v>89</v>
       </c>
@@ -7265,7 +7262,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="F13" s="1">
         <v>88</v>
       </c>
@@ -7276,7 +7273,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="F14" s="1">
         <v>88</v>
       </c>
@@ -7287,7 +7284,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="F15" s="1">
         <v>88</v>
       </c>
@@ -7298,7 +7295,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="F16" s="1">
         <v>88</v>
       </c>
@@ -7309,7 +7306,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F17" s="1">
         <v>88</v>
       </c>
@@ -7320,7 +7317,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="18" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F18" s="1">
         <v>88</v>
       </c>
@@ -7331,7 +7328,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F19" s="1">
         <v>88</v>
       </c>
@@ -7342,7 +7339,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F20" s="1">
         <v>88</v>
       </c>
@@ -7353,7 +7350,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F21" s="1">
         <v>88</v>
       </c>
@@ -7364,7 +7361,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="22" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F22" s="1">
         <v>88</v>
       </c>
@@ -7375,7 +7372,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="23" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F23" s="1">
         <v>88</v>
       </c>
@@ -7386,7 +7383,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="24" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F24" s="1">
         <v>88</v>
       </c>
@@ -7397,7 +7394,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="25" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F25" s="1">
         <v>88</v>
       </c>
@@ -7408,7 +7405,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="26" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F26" s="1">
         <v>88</v>
       </c>
@@ -7419,7 +7416,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="27" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F27" s="1">
         <v>88</v>
       </c>
@@ -7430,7 +7427,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F28" s="1">
         <v>88</v>
       </c>
@@ -7441,7 +7438,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="29" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F29" s="1">
         <v>88</v>
       </c>
@@ -7452,7 +7449,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F30" s="1">
         <v>88</v>
       </c>
@@ -7463,7 +7460,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F31" s="1">
         <v>88</v>
       </c>
@@ -7474,7 +7471,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="32" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F32" s="1">
         <v>88</v>
       </c>
@@ -7485,7 +7482,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="33" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="33" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F33" s="1">
         <v>88</v>
       </c>
@@ -7496,7 +7493,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="34" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="34" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F34" s="1">
         <v>88</v>
       </c>
@@ -7507,7 +7504,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="35" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="35" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F35" s="1">
         <v>88</v>
       </c>
@@ -7518,7 +7515,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="36" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="36" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F36" s="1">
         <v>88</v>
       </c>
@@ -7529,7 +7526,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="37" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="37" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F37" s="1">
         <v>88</v>
       </c>
@@ -7540,7 +7537,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="38" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="38" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F38" s="1">
         <v>88</v>
       </c>
@@ -7551,7 +7548,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="39" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="39" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F39" s="1">
         <v>88</v>
       </c>
@@ -7562,7 +7559,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="40" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="40" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F40" s="1">
         <v>88</v>
       </c>
@@ -7573,7 +7570,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="41" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="41" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F41" s="1">
         <v>88</v>
       </c>
@@ -7584,7 +7581,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="42" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="42" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F42" s="1">
         <v>88</v>
       </c>
@@ -7595,7 +7592,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="43" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="43" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F43" s="1">
         <v>88</v>
       </c>
@@ -7606,7 +7603,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="44" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F44" s="1">
         <v>88</v>
       </c>
@@ -7617,7 +7614,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="45" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="45" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F45" s="1">
         <v>88</v>
       </c>
@@ -7628,7 +7625,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="46" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="46" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F46" s="1">
         <v>88</v>
       </c>
@@ -7639,7 +7636,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="47" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="47" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F47" s="1">
         <v>88</v>
       </c>
@@ -7650,7 +7647,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="48" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="48" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F48" s="1">
         <v>88</v>
       </c>
@@ -7661,7 +7658,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="49" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="49" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F49" s="1">
         <v>88</v>
       </c>
@@ -7672,7 +7669,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="50" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="50" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F50" s="1">
         <v>88</v>
       </c>
@@ -7683,7 +7680,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="51" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="51" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F51" s="1">
         <v>88</v>
       </c>
@@ -7694,7 +7691,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="52" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="52" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F52" s="1">
         <v>88</v>
       </c>
@@ -7705,7 +7702,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="53" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="53" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F53" s="1">
         <v>88</v>
       </c>
@@ -7716,7 +7713,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="54" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="54" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F54" s="1">
         <v>88</v>
       </c>
@@ -7727,7 +7724,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="55" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="55" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F55" s="1">
         <v>88</v>
       </c>
@@ -7738,7 +7735,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="56" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="56" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F56" s="1">
         <v>88</v>
       </c>
@@ -7749,7 +7746,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="57" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="57" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F57" s="1">
         <v>88</v>
       </c>
@@ -7760,7 +7757,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="58" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="58" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F58" s="1">
         <v>88</v>
       </c>
@@ -7771,7 +7768,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="59" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="59" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F59" s="1">
         <v>88</v>
       </c>
@@ -7782,7 +7779,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="60" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="60" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F60" s="1">
         <v>88</v>
       </c>
@@ -7793,7 +7790,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="61" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="61" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F61" s="1">
         <v>88</v>
       </c>
@@ -7804,7 +7801,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="62" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="62" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F62" s="1">
         <v>88</v>
       </c>
@@ -7815,7 +7812,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="63" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="63" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F63" s="1">
         <v>88</v>
       </c>
@@ -7826,7 +7823,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="64" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="64" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F64" s="1">
         <v>88</v>
       </c>
@@ -7837,7 +7834,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.35">
       <c r="F65" s="1">
         <v>88</v>
       </c>
@@ -7848,7 +7845,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.35">
       <c r="F66" s="1">
         <v>88</v>
       </c>
@@ -7859,7 +7856,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A67">
         <v>90</v>
       </c>
@@ -7880,7 +7877,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A68">
         <v>90</v>
       </c>
@@ -7901,7 +7898,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A69">
         <v>90</v>
       </c>
@@ -7922,7 +7919,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A70">
         <v>90</v>
       </c>
@@ -7943,7 +7940,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A71">
         <v>90</v>
       </c>
@@ -7964,7 +7961,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A72">
         <v>90</v>
       </c>
@@ -7985,7 +7982,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A73">
         <v>90</v>
       </c>
@@ -8006,7 +8003,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A74">
         <v>90</v>
       </c>
@@ -8027,7 +8024,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A75">
         <v>80</v>
       </c>
@@ -8048,7 +8045,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.35">
       <c r="F76" s="1">
         <v>88</v>
       </c>
@@ -8059,7 +8056,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.35">
       <c r="F77" s="1">
         <v>88</v>
       </c>
@@ -8070,7 +8067,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.35">
       <c r="F78" s="1">
         <v>88</v>
       </c>
@@ -8081,7 +8078,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.35">
       <c r="F79" s="1">
         <v>88</v>
       </c>
@@ -8092,7 +8089,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.35">
       <c r="F80" s="1">
         <v>88</v>
       </c>
@@ -8103,7 +8100,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="81" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="81" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F81" s="1">
         <v>88</v>
       </c>
@@ -8114,7 +8111,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="82" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="82" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F82" s="1">
         <v>88</v>
       </c>
@@ -8125,7 +8122,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="83" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="83" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F83" s="1">
         <v>88</v>
       </c>
@@ -8136,7 +8133,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="84" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="84" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F84" s="1">
         <v>88</v>
       </c>
@@ -8147,7 +8144,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="85" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="85" spans="6:8" x14ac:dyDescent="0.35">
       <c r="F85" s="1">
         <v>78</v>
       </c>
@@ -8166,18 +8163,18 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{366E84B2-2D8C-4C9C-8D50-353B8B58F7B5}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9" style="1"/>
     <col min="3" max="3" width="19" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9" style="1"/>
-    <col min="5" max="5" width="29.875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.83203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="56.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>324</v>
       </c>
@@ -8203,7 +8200,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>325</v>
       </c>
@@ -8211,16 +8208,16 @@
         <v>305</v>
       </c>
       <c r="C2" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>326</v>
       </c>
       <c r="E2" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="F2">
-        <v>136</v>
+        <v>99</v>
       </c>
       <c r="G2" t="s">
         <v>320</v>

</xml_diff>